<commit_message>
ADD: new logic for discounts
</commit_message>
<xml_diff>
--- a/history_prices/APR/prices_01042026.xlsx
+++ b/history_prices/APR/prices_01042026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\history_prices\APR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0770B66A-C40D-436E-AFF3-3F7501341854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC23B7C-7353-4CC5-AC28-AE87C275A3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="167">
   <si>
     <t>ID</t>
   </si>
@@ -518,6 +518,9 @@
   </si>
   <si>
     <t>200476211</t>
+  </si>
+  <si>
+    <t>ОТСТЪПКА</t>
   </si>
 </sst>
 </file>
@@ -525,9 +528,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="&quot;€&quot;#,##0.000_-"/>
-    <numFmt numFmtId="167" formatCode="&quot;€&quot;#,##0.00_-"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="&quot;€&quot;#,##0.000_-"/>
+    <numFmt numFmtId="166" formatCode="&quot;€&quot;#,##0.00_-"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -558,12 +561,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -866,22 +870,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.5703125" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.28515625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="26.42578125" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="28.140625" customWidth="1"/>
-    <col min="9" max="9" width="27.42578125" customWidth="1"/>
-    <col min="10" max="12" width="23.28515625" customWidth="1"/>
+    <col min="5" max="6" width="26.42578125" customWidth="1"/>
+    <col min="7" max="7" width="23.28515625" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="28.140625" customWidth="1"/>
+    <col min="10" max="10" width="27.42578125" customWidth="1"/>
+    <col min="11" max="13" width="23.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -898,28 +902,31 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -935,23 +942,26 @@
       <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2">
-        <v>1.647</v>
+      <c r="F2" s="5">
+        <v>0</v>
       </c>
       <c r="G2" s="2">
-        <v>0</v>
-      </c>
-      <c r="H2" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
+        <v>1.647</v>
       </c>
       <c r="J2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -967,23 +977,26 @@
       <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="5">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
         <v>1.399</v>
       </c>
-      <c r="G3" s="2">
+      <c r="H3" s="2">
         <v>0.03</v>
       </c>
-      <c r="H3" s="3">
+      <c r="I3" s="3">
         <v>1.429</v>
       </c>
-      <c r="I3" t="s">
-        <v>13</v>
-      </c>
       <c r="J3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -999,23 +1012,26 @@
       <c r="E4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="2">
-        <v>1.647</v>
+      <c r="F4" s="5">
+        <v>0</v>
       </c>
       <c r="G4" s="2">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I4" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3">
+        <v>1.647</v>
       </c>
       <c r="J4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1031,23 +1047,26 @@
       <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="5">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
         <v>1.399</v>
       </c>
-      <c r="G5" s="2">
+      <c r="H5" s="2">
         <v>0.03</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="3">
         <v>1.429</v>
       </c>
-      <c r="I5" t="s">
-        <v>13</v>
-      </c>
       <c r="J5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1063,26 +1082,29 @@
       <c r="E6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="2">
-        <v>1.647</v>
+      <c r="F6" s="5">
+        <v>0</v>
       </c>
       <c r="G6" s="2">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I6" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3">
+        <v>1.647</v>
       </c>
       <c r="J6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" t="s">
         <v>21</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1098,26 +1120,29 @@
       <c r="E7" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
         <v>1.399</v>
       </c>
-      <c r="G7" s="2">
+      <c r="H7" s="2">
         <v>0.03</v>
       </c>
-      <c r="H7" s="3">
+      <c r="I7" s="3">
         <v>1.429</v>
       </c>
-      <c r="I7" t="s">
-        <v>13</v>
-      </c>
       <c r="J7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" t="s">
         <v>21</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -1133,23 +1158,26 @@
       <c r="E8" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="2">
-        <v>1.647</v>
+      <c r="F8" s="5">
+        <v>0</v>
       </c>
       <c r="G8" s="2">
-        <v>0</v>
-      </c>
-      <c r="H8" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I8" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>1.647</v>
       </c>
       <c r="J8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1165,23 +1193,26 @@
       <c r="E9" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
         <v>1.399</v>
       </c>
-      <c r="G9" s="2">
+      <c r="H9" s="2">
         <v>0.03</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="3">
         <v>1.429</v>
       </c>
-      <c r="I9" t="s">
-        <v>13</v>
-      </c>
       <c r="J9" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -1197,23 +1228,26 @@
       <c r="E10" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="2">
-        <v>1.647</v>
+      <c r="F10" s="5">
+        <v>0</v>
       </c>
       <c r="G10" s="2">
+        <v>1.647</v>
+      </c>
+      <c r="H10" s="2">
         <v>0.01</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I10" s="3">
         <v>1.657</v>
       </c>
-      <c r="I10" t="s">
-        <v>13</v>
-      </c>
       <c r="J10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1229,29 +1263,32 @@
       <c r="E11" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="2">
-        <v>1.647</v>
+      <c r="F11" s="5">
+        <v>0</v>
       </c>
       <c r="G11" s="2">
-        <v>0</v>
-      </c>
-      <c r="H11" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I11" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" s="3">
+        <v>1.647</v>
       </c>
       <c r="J11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" t="s">
         <v>30</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>31</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -1267,29 +1304,32 @@
       <c r="E12" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="5">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2">
         <v>1.399</v>
       </c>
-      <c r="G12" s="2">
+      <c r="H12" s="2">
         <v>0.03</v>
       </c>
-      <c r="H12" s="3">
+      <c r="I12" s="3">
         <v>1.429</v>
       </c>
-      <c r="I12" t="s">
-        <v>13</v>
-      </c>
       <c r="J12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" t="s">
         <v>30</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>31</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -1305,23 +1345,26 @@
       <c r="E13" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="2">
-        <v>1.647</v>
+      <c r="F13" s="5">
+        <v>0</v>
       </c>
       <c r="G13" s="2">
-        <v>0</v>
-      </c>
-      <c r="H13" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I13" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>1.647</v>
       </c>
       <c r="J13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -1337,23 +1380,26 @@
       <c r="E14" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="5">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2">
         <v>1.399</v>
       </c>
-      <c r="G14" s="2">
+      <c r="H14" s="2">
         <v>0.04</v>
       </c>
-      <c r="H14" s="3">
+      <c r="I14" s="3">
         <v>1.4390000000000001</v>
       </c>
-      <c r="I14" t="s">
-        <v>13</v>
-      </c>
       <c r="J14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -1369,23 +1415,26 @@
       <c r="E15" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="2">
-        <v>1.647</v>
+      <c r="F15" s="5">
+        <v>0</v>
       </c>
       <c r="G15" s="2">
-        <v>0</v>
-      </c>
-      <c r="H15" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I15" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3">
+        <v>1.647</v>
       </c>
       <c r="J15" t="s">
+        <v>13</v>
+      </c>
+      <c r="K15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -1401,23 +1450,26 @@
       <c r="E16" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
         <v>1.399</v>
       </c>
-      <c r="G16" s="2">
+      <c r="H16" s="2">
         <v>0.04</v>
       </c>
-      <c r="H16" s="3">
+      <c r="I16" s="3">
         <v>1.4390000000000001</v>
       </c>
-      <c r="I16" t="s">
-        <v>13</v>
-      </c>
       <c r="J16" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -1433,23 +1485,26 @@
       <c r="E17" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="2">
-        <v>1.647</v>
+      <c r="F17" s="5">
+        <v>0</v>
       </c>
       <c r="G17" s="2">
-        <v>0</v>
-      </c>
-      <c r="H17" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I17" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3">
+        <v>1.647</v>
       </c>
       <c r="J17" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -1465,23 +1520,26 @@
       <c r="E18" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="5">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2">
         <v>1.399</v>
       </c>
-      <c r="G18" s="2">
+      <c r="H18" s="2">
         <v>0.04</v>
       </c>
-      <c r="H18" s="3">
+      <c r="I18" s="3">
         <v>1.4390000000000001</v>
       </c>
-      <c r="I18" t="s">
-        <v>13</v>
-      </c>
       <c r="J18" t="s">
+        <v>13</v>
+      </c>
+      <c r="K18" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -1497,26 +1555,29 @@
       <c r="E19" t="s">
         <v>12</v>
       </c>
-      <c r="F19" s="2">
-        <v>1.647</v>
+      <c r="F19" s="5">
+        <v>0</v>
       </c>
       <c r="G19" s="2">
-        <v>0</v>
-      </c>
-      <c r="H19" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I19" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H19" s="2">
+        <v>0</v>
+      </c>
+      <c r="I19" s="3">
+        <v>1.647</v>
       </c>
       <c r="J19" t="s">
+        <v>13</v>
+      </c>
+      <c r="K19" t="s">
         <v>44</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>46</v>
       </c>
@@ -1532,26 +1593,29 @@
       <c r="E20" t="s">
         <v>47</v>
       </c>
-      <c r="F20" s="2">
-        <v>1.647</v>
+      <c r="F20" s="5">
+        <v>0</v>
       </c>
       <c r="G20" s="2">
+        <v>1.647</v>
+      </c>
+      <c r="H20" s="2">
         <v>0.09</v>
       </c>
-      <c r="H20" s="3">
+      <c r="I20" s="3">
         <v>1.7370000000000001</v>
       </c>
-      <c r="I20" t="s">
-        <v>13</v>
-      </c>
       <c r="J20" t="s">
+        <v>13</v>
+      </c>
+      <c r="K20" t="s">
         <v>44</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -1567,26 +1631,29 @@
       <c r="E21" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
         <v>1.399</v>
       </c>
-      <c r="G21" s="2">
+      <c r="H21" s="2">
         <v>0.03</v>
       </c>
-      <c r="H21" s="3">
+      <c r="I21" s="3">
         <v>1.429</v>
       </c>
-      <c r="I21" t="s">
-        <v>13</v>
-      </c>
       <c r="J21" t="s">
+        <v>13</v>
+      </c>
+      <c r="K21" t="s">
         <v>44</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -1602,26 +1669,29 @@
       <c r="E22" t="s">
         <v>50</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2">
         <v>1.61</v>
       </c>
-      <c r="G22" s="2">
+      <c r="H22" s="2">
         <v>0.09</v>
       </c>
-      <c r="H22" s="3">
+      <c r="I22" s="3">
         <v>1.7</v>
       </c>
-      <c r="I22" t="s">
-        <v>13</v>
-      </c>
       <c r="J22" t="s">
+        <v>13</v>
+      </c>
+      <c r="K22" t="s">
         <v>44</v>
       </c>
-      <c r="K22" t="s">
+      <c r="L22" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -1637,26 +1707,29 @@
       <c r="E23" t="s">
         <v>12</v>
       </c>
-      <c r="F23" s="2">
-        <v>1.647</v>
+      <c r="F23" s="5">
+        <v>0</v>
       </c>
       <c r="G23" s="2">
-        <v>0</v>
-      </c>
-      <c r="H23" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I23" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H23" s="2">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3">
+        <v>1.647</v>
       </c>
       <c r="J23" t="s">
+        <v>13</v>
+      </c>
+      <c r="K23" t="s">
         <v>52</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -1672,26 +1745,29 @@
       <c r="E24" t="s">
         <v>47</v>
       </c>
-      <c r="F24" s="2">
-        <v>1.647</v>
+      <c r="F24" s="5">
+        <v>0</v>
       </c>
       <c r="G24" s="2">
+        <v>1.647</v>
+      </c>
+      <c r="H24" s="2">
         <v>0.09</v>
       </c>
-      <c r="H24" s="3">
+      <c r="I24" s="3">
         <v>1.7370000000000001</v>
       </c>
-      <c r="I24" t="s">
-        <v>13</v>
-      </c>
       <c r="J24" t="s">
+        <v>13</v>
+      </c>
+      <c r="K24" t="s">
         <v>52</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -1707,26 +1783,29 @@
       <c r="E25" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="5">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2">
         <v>1.399</v>
       </c>
-      <c r="G25" s="2">
+      <c r="H25" s="2">
         <v>0.03</v>
       </c>
-      <c r="H25" s="3">
+      <c r="I25" s="3">
         <v>1.429</v>
       </c>
-      <c r="I25" t="s">
-        <v>13</v>
-      </c>
       <c r="J25" t="s">
+        <v>13</v>
+      </c>
+      <c r="K25" t="s">
         <v>52</v>
       </c>
-      <c r="K25" t="s">
+      <c r="L25" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>56</v>
       </c>
@@ -1742,26 +1821,29 @@
       <c r="E26" t="s">
         <v>50</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="5">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
         <v>1.61</v>
       </c>
-      <c r="G26" s="2">
+      <c r="H26" s="2">
         <v>0.09</v>
       </c>
-      <c r="H26" s="3">
+      <c r="I26" s="3">
         <v>1.7</v>
       </c>
-      <c r="I26" t="s">
-        <v>13</v>
-      </c>
       <c r="J26" t="s">
+        <v>13</v>
+      </c>
+      <c r="K26" t="s">
         <v>52</v>
       </c>
-      <c r="K26" t="s">
+      <c r="L26" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>57</v>
       </c>
@@ -1777,23 +1859,26 @@
       <c r="E27" t="s">
         <v>12</v>
       </c>
-      <c r="F27" s="2">
-        <v>1.647</v>
+      <c r="F27" s="5">
+        <v>0</v>
       </c>
       <c r="G27" s="2">
-        <v>0</v>
-      </c>
-      <c r="H27" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I27" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H27" s="2">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3">
+        <v>1.647</v>
       </c>
       <c r="J27" t="s">
+        <v>13</v>
+      </c>
+      <c r="K27" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -1809,23 +1894,26 @@
       <c r="E28" t="s">
         <v>16</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="5">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2">
         <v>1.399</v>
       </c>
-      <c r="G28" s="2">
+      <c r="H28" s="2">
         <v>0.04</v>
       </c>
-      <c r="H28" s="3">
+      <c r="I28" s="3">
         <v>1.4390000000000001</v>
       </c>
-      <c r="I28" t="s">
-        <v>13</v>
-      </c>
       <c r="J28" t="s">
+        <v>13</v>
+      </c>
+      <c r="K28" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>60</v>
       </c>
@@ -1841,26 +1929,29 @@
       <c r="E29" t="s">
         <v>12</v>
       </c>
-      <c r="F29" s="2">
-        <v>1.647</v>
+      <c r="F29" s="5">
+        <v>0</v>
       </c>
       <c r="G29" s="2">
-        <v>0</v>
-      </c>
-      <c r="H29" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I29" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H29" s="2">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3">
+        <v>1.647</v>
       </c>
       <c r="J29" t="s">
+        <v>13</v>
+      </c>
+      <c r="K29" t="s">
         <v>61</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -1876,26 +1967,29 @@
       <c r="E30" t="s">
         <v>16</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="5">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2">
         <v>1.399</v>
       </c>
-      <c r="G30" s="2">
+      <c r="H30" s="2">
         <v>0.02</v>
       </c>
-      <c r="H30" s="3">
+      <c r="I30" s="3">
         <v>1.419</v>
       </c>
-      <c r="I30" t="s">
-        <v>13</v>
-      </c>
       <c r="J30" t="s">
+        <v>13</v>
+      </c>
+      <c r="K30" t="s">
         <v>61</v>
       </c>
-      <c r="K30" t="s">
+      <c r="L30" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>64</v>
       </c>
@@ -1911,23 +2005,26 @@
       <c r="E31" t="s">
         <v>12</v>
       </c>
-      <c r="F31" s="2">
-        <v>1.647</v>
+      <c r="F31" s="5">
+        <v>0</v>
       </c>
       <c r="G31" s="2">
-        <v>0</v>
-      </c>
-      <c r="H31" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I31" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H31" s="2">
+        <v>0</v>
+      </c>
+      <c r="I31" s="3">
+        <v>1.647</v>
       </c>
       <c r="J31" t="s">
+        <v>13</v>
+      </c>
+      <c r="K31" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>66</v>
       </c>
@@ -1943,23 +2040,26 @@
       <c r="E32" t="s">
         <v>16</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="5">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2">
         <v>1.399</v>
       </c>
-      <c r="G32" s="2">
+      <c r="H32" s="2">
         <v>0.03</v>
       </c>
-      <c r="H32" s="3">
+      <c r="I32" s="3">
         <v>1.429</v>
       </c>
-      <c r="I32" t="s">
-        <v>13</v>
-      </c>
       <c r="J32" t="s">
+        <v>13</v>
+      </c>
+      <c r="K32" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>67</v>
       </c>
@@ -1975,23 +2075,26 @@
       <c r="E33" t="s">
         <v>12</v>
       </c>
-      <c r="F33" s="2">
-        <v>1.647</v>
+      <c r="F33" s="5">
+        <v>0</v>
       </c>
       <c r="G33" s="2">
-        <v>0</v>
-      </c>
-      <c r="H33" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I33" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H33" s="2">
+        <v>0</v>
+      </c>
+      <c r="I33" s="3">
+        <v>1.647</v>
       </c>
       <c r="J33" t="s">
+        <v>13</v>
+      </c>
+      <c r="K33" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -2007,26 +2110,29 @@
       <c r="E34" t="s">
         <v>12</v>
       </c>
-      <c r="F34" s="2">
-        <v>1.647</v>
+      <c r="F34" s="5">
+        <v>0</v>
       </c>
       <c r="G34" s="2">
-        <v>0</v>
-      </c>
-      <c r="H34" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I34" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H34" s="2">
+        <v>0</v>
+      </c>
+      <c r="I34" s="3">
+        <v>1.647</v>
       </c>
       <c r="J34" t="s">
+        <v>13</v>
+      </c>
+      <c r="K34" t="s">
         <v>70</v>
       </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>72</v>
       </c>
@@ -2042,26 +2148,29 @@
       <c r="E35" t="s">
         <v>16</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="5">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2">
         <v>1.399</v>
       </c>
-      <c r="G35" s="2">
+      <c r="H35" s="2">
         <v>0.03</v>
       </c>
-      <c r="H35" s="3">
+      <c r="I35" s="3">
         <v>1.429</v>
       </c>
-      <c r="I35" t="s">
-        <v>13</v>
-      </c>
       <c r="J35" t="s">
+        <v>13</v>
+      </c>
+      <c r="K35" t="s">
         <v>70</v>
       </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -2077,23 +2186,26 @@
       <c r="E36" t="s">
         <v>12</v>
       </c>
-      <c r="F36" s="2">
-        <v>1.647</v>
+      <c r="F36" s="5">
+        <v>0</v>
       </c>
       <c r="G36" s="2">
-        <v>0</v>
-      </c>
-      <c r="H36" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I36" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H36" s="2">
+        <v>0</v>
+      </c>
+      <c r="I36" s="3">
+        <v>1.647</v>
       </c>
       <c r="J36" t="s">
+        <v>13</v>
+      </c>
+      <c r="K36" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -2109,23 +2221,26 @@
       <c r="E37" t="s">
         <v>12</v>
       </c>
-      <c r="F37" s="2">
-        <v>1.647</v>
+      <c r="F37" s="5">
+        <v>0</v>
       </c>
       <c r="G37" s="2">
-        <v>0</v>
-      </c>
-      <c r="H37" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I37" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H37" s="2">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3">
+        <v>1.647</v>
       </c>
       <c r="J37" t="s">
+        <v>13</v>
+      </c>
+      <c r="K37" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>77</v>
       </c>
@@ -2141,23 +2256,26 @@
       <c r="E38" t="s">
         <v>16</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="5">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2">
         <v>1.399</v>
       </c>
-      <c r="G38" s="2">
+      <c r="H38" s="2">
         <v>0.03</v>
       </c>
-      <c r="H38" s="3">
+      <c r="I38" s="3">
         <v>1.429</v>
       </c>
-      <c r="I38" t="s">
-        <v>13</v>
-      </c>
       <c r="J38" t="s">
+        <v>13</v>
+      </c>
+      <c r="K38" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -2173,26 +2291,29 @@
       <c r="E39" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="2">
-        <v>1.647</v>
+      <c r="F39" s="5">
+        <v>0</v>
       </c>
       <c r="G39" s="2">
-        <v>0</v>
-      </c>
-      <c r="H39" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I39" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H39" s="2">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3">
+        <v>1.647</v>
       </c>
       <c r="J39" t="s">
+        <v>13</v>
+      </c>
+      <c r="K39" t="s">
         <v>79</v>
       </c>
-      <c r="K39" t="s">
+      <c r="L39" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>81</v>
       </c>
@@ -2208,26 +2329,29 @@
       <c r="E40" t="s">
         <v>47</v>
       </c>
-      <c r="F40" s="2">
-        <v>1.647</v>
+      <c r="F40" s="5">
+        <v>0</v>
       </c>
       <c r="G40" s="2">
+        <v>1.647</v>
+      </c>
+      <c r="H40" s="2">
         <v>0.09</v>
       </c>
-      <c r="H40" s="3">
+      <c r="I40" s="3">
         <v>1.7370000000000001</v>
       </c>
-      <c r="I40" t="s">
-        <v>13</v>
-      </c>
       <c r="J40" t="s">
+        <v>13</v>
+      </c>
+      <c r="K40" t="s">
         <v>79</v>
       </c>
-      <c r="K40" t="s">
+      <c r="L40" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>82</v>
       </c>
@@ -2243,26 +2367,29 @@
       <c r="E41" t="s">
         <v>16</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="5">
+        <v>0</v>
+      </c>
+      <c r="G41" s="2">
         <v>1.399</v>
       </c>
-      <c r="G41" s="2">
+      <c r="H41" s="2">
         <v>0.03</v>
       </c>
-      <c r="H41" s="3">
+      <c r="I41" s="3">
         <v>1.429</v>
       </c>
-      <c r="I41" t="s">
-        <v>13</v>
-      </c>
       <c r="J41" t="s">
+        <v>13</v>
+      </c>
+      <c r="K41" t="s">
         <v>79</v>
       </c>
-      <c r="K41" t="s">
+      <c r="L41" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>83</v>
       </c>
@@ -2278,26 +2405,29 @@
       <c r="E42" t="s">
         <v>50</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="5">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2">
         <v>1.61</v>
       </c>
-      <c r="G42" s="2">
+      <c r="H42" s="2">
         <v>0.09</v>
       </c>
-      <c r="H42" s="3">
+      <c r="I42" s="3">
         <v>1.7</v>
       </c>
-      <c r="I42" t="s">
-        <v>13</v>
-      </c>
       <c r="J42" t="s">
+        <v>13</v>
+      </c>
+      <c r="K42" t="s">
         <v>79</v>
       </c>
-      <c r="K42" t="s">
+      <c r="L42" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>84</v>
       </c>
@@ -2313,23 +2443,26 @@
       <c r="E43" t="s">
         <v>12</v>
       </c>
-      <c r="F43" s="2">
-        <v>1.647</v>
+      <c r="F43" s="5">
+        <v>0</v>
       </c>
       <c r="G43" s="2">
-        <v>0</v>
-      </c>
-      <c r="H43" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I43" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H43" s="2">
+        <v>0</v>
+      </c>
+      <c r="I43" s="3">
+        <v>1.647</v>
       </c>
       <c r="J43" t="s">
+        <v>13</v>
+      </c>
+      <c r="K43" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>86</v>
       </c>
@@ -2345,23 +2478,26 @@
       <c r="E44" t="s">
         <v>16</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="5">
+        <v>0</v>
+      </c>
+      <c r="G44" s="2">
         <v>1.399</v>
       </c>
-      <c r="G44" s="2">
+      <c r="H44" s="2">
         <v>0.03</v>
       </c>
-      <c r="H44" s="3">
+      <c r="I44" s="3">
         <v>1.429</v>
       </c>
-      <c r="I44" t="s">
-        <v>13</v>
-      </c>
       <c r="J44" t="s">
+        <v>13</v>
+      </c>
+      <c r="K44" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>87</v>
       </c>
@@ -2377,26 +2513,29 @@
       <c r="E45" t="s">
         <v>12</v>
       </c>
-      <c r="F45" s="2">
-        <v>1.647</v>
+      <c r="F45" s="5">
+        <v>0</v>
       </c>
       <c r="G45" s="2">
-        <v>0</v>
-      </c>
-      <c r="H45" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I45" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H45" s="2">
+        <v>0</v>
+      </c>
+      <c r="I45" s="3">
+        <v>1.647</v>
       </c>
       <c r="J45" t="s">
+        <v>13</v>
+      </c>
+      <c r="K45" t="s">
         <v>88</v>
       </c>
-      <c r="K45" t="s">
+      <c r="L45" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>90</v>
       </c>
@@ -2412,26 +2551,29 @@
       <c r="E46" t="s">
         <v>47</v>
       </c>
-      <c r="F46" s="2">
-        <v>1.647</v>
+      <c r="F46" s="5">
+        <v>0</v>
       </c>
       <c r="G46" s="2">
+        <v>1.647</v>
+      </c>
+      <c r="H46" s="2">
         <v>0.09</v>
       </c>
-      <c r="H46" s="3">
+      <c r="I46" s="3">
         <v>1.7370000000000001</v>
       </c>
-      <c r="I46" t="s">
-        <v>13</v>
-      </c>
       <c r="J46" t="s">
+        <v>13</v>
+      </c>
+      <c r="K46" t="s">
         <v>88</v>
       </c>
-      <c r="K46" t="s">
+      <c r="L46" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>91</v>
       </c>
@@ -2447,26 +2589,29 @@
       <c r="E47" t="s">
         <v>16</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="5">
+        <v>0</v>
+      </c>
+      <c r="G47" s="2">
         <v>1.399</v>
       </c>
-      <c r="G47" s="2">
+      <c r="H47" s="2">
         <v>0.03</v>
       </c>
-      <c r="H47" s="3">
+      <c r="I47" s="3">
         <v>1.429</v>
       </c>
-      <c r="I47" t="s">
-        <v>13</v>
-      </c>
       <c r="J47" t="s">
+        <v>13</v>
+      </c>
+      <c r="K47" t="s">
         <v>88</v>
       </c>
-      <c r="K47" t="s">
+      <c r="L47" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>92</v>
       </c>
@@ -2482,26 +2627,29 @@
       <c r="E48" t="s">
         <v>50</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="5">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2">
         <v>1.61</v>
       </c>
-      <c r="G48" s="2">
+      <c r="H48" s="2">
         <v>0.09</v>
       </c>
-      <c r="H48" s="3">
+      <c r="I48" s="3">
         <v>1.7</v>
       </c>
-      <c r="I48" t="s">
-        <v>13</v>
-      </c>
       <c r="J48" t="s">
+        <v>13</v>
+      </c>
+      <c r="K48" t="s">
         <v>88</v>
       </c>
-      <c r="K48" t="s">
+      <c r="L48" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>93</v>
       </c>
@@ -2517,26 +2665,29 @@
       <c r="E49" t="s">
         <v>12</v>
       </c>
-      <c r="F49" s="2">
-        <v>1.647</v>
+      <c r="F49" s="5">
+        <v>0</v>
       </c>
       <c r="G49" s="2">
-        <v>0</v>
-      </c>
-      <c r="H49" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I49" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H49" s="2">
+        <v>0</v>
+      </c>
+      <c r="I49" s="3">
+        <v>1.647</v>
       </c>
       <c r="J49" t="s">
+        <v>13</v>
+      </c>
+      <c r="K49" t="s">
         <v>94</v>
       </c>
-      <c r="K49" t="s">
+      <c r="L49" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>96</v>
       </c>
@@ -2552,26 +2703,29 @@
       <c r="E50" t="s">
         <v>47</v>
       </c>
-      <c r="F50" s="2">
-        <v>1.647</v>
+      <c r="F50" s="5">
+        <v>0</v>
       </c>
       <c r="G50" s="2">
+        <v>1.647</v>
+      </c>
+      <c r="H50" s="2">
         <v>0.09</v>
       </c>
-      <c r="H50" s="3">
+      <c r="I50" s="3">
         <v>1.7370000000000001</v>
       </c>
-      <c r="I50" t="s">
-        <v>13</v>
-      </c>
       <c r="J50" t="s">
+        <v>13</v>
+      </c>
+      <c r="K50" t="s">
         <v>94</v>
       </c>
-      <c r="K50" t="s">
+      <c r="L50" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>97</v>
       </c>
@@ -2587,26 +2741,29 @@
       <c r="E51" t="s">
         <v>16</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="5">
+        <v>0</v>
+      </c>
+      <c r="G51" s="2">
         <v>1.399</v>
       </c>
-      <c r="G51" s="2">
+      <c r="H51" s="2">
         <v>0.03</v>
       </c>
-      <c r="H51" s="3">
+      <c r="I51" s="3">
         <v>1.429</v>
       </c>
-      <c r="I51" t="s">
-        <v>13</v>
-      </c>
       <c r="J51" t="s">
+        <v>13</v>
+      </c>
+      <c r="K51" t="s">
         <v>94</v>
       </c>
-      <c r="K51" t="s">
+      <c r="L51" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>98</v>
       </c>
@@ -2622,26 +2779,29 @@
       <c r="E52" t="s">
         <v>50</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="5">
+        <v>0</v>
+      </c>
+      <c r="G52" s="2">
         <v>1.61</v>
       </c>
-      <c r="G52" s="2">
+      <c r="H52" s="2">
         <v>0.09</v>
       </c>
-      <c r="H52" s="3">
+      <c r="I52" s="3">
         <v>1.7</v>
       </c>
-      <c r="I52" t="s">
-        <v>13</v>
-      </c>
       <c r="J52" t="s">
+        <v>13</v>
+      </c>
+      <c r="K52" t="s">
         <v>94</v>
       </c>
-      <c r="K52" t="s">
+      <c r="L52" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>99</v>
       </c>
@@ -2657,17 +2817,20 @@
       <c r="E53" t="s">
         <v>12</v>
       </c>
-      <c r="F53" s="2">
-        <v>1.647</v>
+      <c r="F53" s="5">
+        <v>0</v>
       </c>
       <c r="G53" s="2">
-        <v>0</v>
-      </c>
-      <c r="H53" s="3">
-        <v>1.647</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.647</v>
+      </c>
+      <c r="H53" s="2">
+        <v>0</v>
+      </c>
+      <c r="I53" s="3">
+        <v>1.647</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>100</v>
       </c>
@@ -2683,17 +2846,20 @@
       <c r="E54" t="s">
         <v>12</v>
       </c>
-      <c r="F54" s="2">
-        <v>1.647</v>
+      <c r="F54" s="5">
+        <v>0</v>
       </c>
       <c r="G54" s="2">
-        <v>0</v>
-      </c>
-      <c r="H54" s="3">
-        <v>1.647</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.647</v>
+      </c>
+      <c r="H54" s="2">
+        <v>0</v>
+      </c>
+      <c r="I54" s="3">
+        <v>1.647</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>101</v>
       </c>
@@ -2709,17 +2875,20 @@
       <c r="E55" t="s">
         <v>12</v>
       </c>
-      <c r="F55" s="2">
-        <v>1.647</v>
+      <c r="F55" s="5">
+        <v>0</v>
       </c>
       <c r="G55" s="2">
-        <v>0</v>
-      </c>
-      <c r="H55" s="3">
-        <v>1.647</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.647</v>
+      </c>
+      <c r="H55" s="2">
+        <v>0</v>
+      </c>
+      <c r="I55" s="3">
+        <v>1.647</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>102</v>
       </c>
@@ -2735,17 +2904,20 @@
       <c r="E56" t="s">
         <v>12</v>
       </c>
-      <c r="F56" s="2">
-        <v>1.647</v>
+      <c r="F56" s="5">
+        <v>0</v>
       </c>
       <c r="G56" s="2">
-        <v>0</v>
-      </c>
-      <c r="H56" s="3">
-        <v>1.647</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.647</v>
+      </c>
+      <c r="H56" s="2">
+        <v>0</v>
+      </c>
+      <c r="I56" s="3">
+        <v>1.647</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>103</v>
       </c>
@@ -2761,17 +2933,20 @@
       <c r="E57" t="s">
         <v>12</v>
       </c>
-      <c r="F57" s="2">
-        <v>1.647</v>
+      <c r="F57" s="5">
+        <v>0</v>
       </c>
       <c r="G57" s="2">
-        <v>0</v>
-      </c>
-      <c r="H57" s="3">
-        <v>1.647</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.647</v>
+      </c>
+      <c r="H57" s="2">
+        <v>0</v>
+      </c>
+      <c r="I57" s="3">
+        <v>1.647</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>104</v>
       </c>
@@ -2787,17 +2962,20 @@
       <c r="E58" t="s">
         <v>16</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="5">
+        <v>0</v>
+      </c>
+      <c r="G58" s="2">
         <v>1.399</v>
       </c>
-      <c r="G58" s="2">
+      <c r="H58" s="2">
         <v>0.04</v>
       </c>
-      <c r="H58" s="3">
+      <c r="I58" s="3">
         <v>1.4390000000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>105</v>
       </c>
@@ -2813,17 +2991,20 @@
       <c r="E59" t="s">
         <v>16</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="5">
+        <v>0</v>
+      </c>
+      <c r="G59" s="2">
         <v>1.399</v>
       </c>
-      <c r="G59" s="2">
+      <c r="H59" s="2">
         <v>0.03</v>
       </c>
-      <c r="H59" s="3">
+      <c r="I59" s="3">
         <v>1.429</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>106</v>
       </c>
@@ -2839,17 +3020,20 @@
       <c r="E60" t="s">
         <v>12</v>
       </c>
-      <c r="F60" s="2">
-        <v>1.647</v>
+      <c r="F60" s="5">
+        <v>0</v>
       </c>
       <c r="G60" s="2">
-        <v>0</v>
-      </c>
-      <c r="H60" s="3">
-        <v>1.647</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.647</v>
+      </c>
+      <c r="H60" s="2">
+        <v>0</v>
+      </c>
+      <c r="I60" s="3">
+        <v>1.647</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>107</v>
       </c>
@@ -2865,17 +3049,20 @@
       <c r="E61" t="s">
         <v>16</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="5">
+        <v>0</v>
+      </c>
+      <c r="G61" s="2">
         <v>1.399</v>
       </c>
-      <c r="G61" s="2">
+      <c r="H61" s="2">
         <v>0.03</v>
       </c>
-      <c r="H61" s="3">
+      <c r="I61" s="3">
         <v>1.429</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>108</v>
       </c>
@@ -2891,17 +3078,20 @@
       <c r="E62" t="s">
         <v>12</v>
       </c>
-      <c r="F62" s="2">
-        <v>1.647</v>
+      <c r="F62" s="5">
+        <v>0</v>
       </c>
       <c r="G62" s="2">
-        <v>0</v>
-      </c>
-      <c r="H62" s="3">
-        <v>1.647</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.647</v>
+      </c>
+      <c r="H62" s="2">
+        <v>0</v>
+      </c>
+      <c r="I62" s="3">
+        <v>1.647</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>109</v>
       </c>
@@ -2917,17 +3107,20 @@
       <c r="E63" t="s">
         <v>16</v>
       </c>
-      <c r="F63" s="2">
+      <c r="F63" s="5">
+        <v>0</v>
+      </c>
+      <c r="G63" s="2">
         <v>1.399</v>
       </c>
-      <c r="G63" s="2">
+      <c r="H63" s="2">
         <v>0.03</v>
       </c>
-      <c r="H63" s="3">
+      <c r="I63" s="3">
         <v>1.429</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>110</v>
       </c>
@@ -2943,17 +3136,20 @@
       <c r="E64" t="s">
         <v>16</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="5">
+        <v>0</v>
+      </c>
+      <c r="G64" s="2">
         <v>1.399</v>
       </c>
-      <c r="G64" s="2">
+      <c r="H64" s="2">
         <v>0.02</v>
       </c>
-      <c r="H64" s="3">
+      <c r="I64" s="3">
         <v>1.419</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>111</v>
       </c>
@@ -2969,17 +3165,20 @@
       <c r="E65" t="s">
         <v>16</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F65" s="5">
+        <v>0</v>
+      </c>
+      <c r="G65" s="2">
         <v>1.399</v>
       </c>
-      <c r="G65" s="2">
+      <c r="H65" s="2">
         <v>0.02</v>
       </c>
-      <c r="H65" s="3">
+      <c r="I65" s="3">
         <v>1.419</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>112</v>
       </c>
@@ -2995,17 +3194,20 @@
       <c r="E66" t="s">
         <v>16</v>
       </c>
-      <c r="F66" s="2">
+      <c r="F66" s="5">
+        <v>0</v>
+      </c>
+      <c r="G66" s="2">
         <v>1.399</v>
       </c>
-      <c r="G66" s="2">
+      <c r="H66" s="2">
         <v>0.03</v>
       </c>
-      <c r="H66" s="3">
+      <c r="I66" s="3">
         <v>1.429</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>113</v>
       </c>
@@ -3021,23 +3223,26 @@
       <c r="E67" t="s">
         <v>12</v>
       </c>
-      <c r="F67" s="2">
-        <v>1.647</v>
+      <c r="F67" s="5">
+        <v>0</v>
       </c>
       <c r="G67" s="2">
-        <v>0</v>
-      </c>
-      <c r="H67" s="3">
-        <v>1.647</v>
-      </c>
-      <c r="I67" t="s">
-        <v>13</v>
+        <v>1.647</v>
+      </c>
+      <c r="H67" s="2">
+        <v>0</v>
+      </c>
+      <c r="I67" s="3">
+        <v>1.647</v>
       </c>
       <c r="J67" t="s">
+        <v>13</v>
+      </c>
+      <c r="K67" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>116</v>
       </c>
@@ -3053,19 +3258,22 @@
       <c r="E68" t="s">
         <v>16</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="5">
+        <v>0</v>
+      </c>
+      <c r="G68" s="2">
         <v>1.399</v>
       </c>
-      <c r="G68" s="2">
+      <c r="H68" s="2">
         <v>0.02</v>
       </c>
-      <c r="H68" s="3">
+      <c r="I68" s="3">
         <v>1.419</v>
       </c>
-      <c r="I68" t="s">
-        <v>13</v>
-      </c>
       <c r="J68" t="s">
+        <v>13</v>
+      </c>
+      <c r="K68" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>